<commit_message>
Visual Logo - Dark Light Mode
</commit_message>
<xml_diff>
--- a/Data/Proyecciones_Multimodelo.xlsx
+++ b/Data/Proyecciones_Multimodelo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5f15395a9ed9a48f/Imágenes/Proyectos/Indicadores/Modelo_Prospectivo/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="769" documentId="8_{44BC8EE8-0004-4F82-B9F9-910542D6C047}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{667BC7F2-5C26-4C08-9F6F-6D8E2B237192}"/>
+  <xr:revisionPtr revIDLastSave="779" documentId="8_{44BC8EE8-0004-4F82-B9F9-910542D6C047}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{90EDE26E-CD4B-4997-9504-0F4F4C9EC229}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E56FC6A2-DA73-40EE-B621-BA207259297A}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Proyecciones" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Proyecciones!$A$1:$I$466</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Proyecciones!$A$1:$K$466</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -668,7 +668,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52F5ABF9-7414-4626-A0F7-29EA0F0D3250}">
-  <dimension ref="A1:I466"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:K466"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="17.88671875" bestFit="1" customWidth="1"/>
@@ -703,7 +704,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>109</v>
       </c>
@@ -732,7 +733,7 @@
         <v>96.466210501716631</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>109</v>
       </c>
@@ -761,7 +762,7 @@
         <v>98.817673270209056</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>109</v>
       </c>
@@ -790,7 +791,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>109</v>
       </c>
@@ -819,7 +820,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>109</v>
       </c>
@@ -848,7 +849,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>148</v>
       </c>
@@ -877,7 +878,7 @@
         <v>6.4632000000000014</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>148</v>
       </c>
@@ -906,7 +907,7 @@
         <v>6.6767605714285727</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>148</v>
       </c>
@@ -935,7 +936,7 @@
         <v>6.8921245714285728</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>148</v>
       </c>
@@ -964,7 +965,7 @@
         <v>7.1092920000000008</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>148</v>
       </c>
@@ -993,7 +994,7 @@
         <v>7.3282628571428594</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>148</v>
       </c>
@@ -1022,7 +1023,7 @@
         <v>7.5490371428571432</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>148</v>
       </c>
@@ -1051,7 +1052,7 @@
         <v>7.7716148571428576</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>148</v>
       </c>
@@ -1080,7 +1081,7 @@
         <v>7.9959960000000017</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>148</v>
       </c>
@@ -1109,7 +1110,7 @@
         <v>8.2221805714285736</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>148</v>
       </c>
@@ -1138,7 +1139,7 @@
         <v>8.4501685714285717</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>148</v>
       </c>
@@ -1167,7 +1168,7 @@
         <v>6.1899902761070864</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>148</v>
       </c>
@@ -1196,7 +1197,7 @@
         <v>6.3279819822962171</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>148</v>
       </c>
@@ -1225,7 +1226,7 @@
         <v>6.4686394813710644</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>148</v>
       </c>
@@ -1254,7 +1255,7 @@
         <v>6.6119865461157588</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>148</v>
       </c>
@@ -1283,7 +1284,7 @@
         <v>6.7580469493144291</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>148</v>
       </c>
@@ -1312,7 +1313,7 @@
         <v>6.906844463751205</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>148</v>
       </c>
@@ -1341,7 +1342,7 @@
         <v>7.0584028622102162</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>148</v>
       </c>
@@ -1370,7 +1371,7 @@
         <v>7.2127459174755941</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>148</v>
       </c>
@@ -1399,7 +1400,7 @@
         <v>7.3698974023314676</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>148</v>
       </c>
@@ -1428,7 +1429,7 @@
         <v>7.5298810895619628</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>148</v>
       </c>
@@ -1457,7 +1458,7 @@
         <v>6.4272000000000009</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>148</v>
       </c>
@@ -1486,7 +1487,7 @@
         <v>6.6531160800000002</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>148</v>
       </c>
@@ -1515,7 +1516,7 @@
         <v>6.8868026448000004</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>148</v>
       </c>
@@ -1544,7 +1545,7 @@
         <v>7.1285225990160006</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>148</v>
       </c>
@@ -1573,7 +1574,7 @@
         <v>7.3785476281046396</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>148</v>
       </c>
@@ -1602,7 +1603,7 @@
         <v>7.6371584885994839</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>148</v>
       </c>
@@ -1631,7 +1632,7 @@
         <v>7.9046453078587247</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>148</v>
       </c>
@@ -1660,7 +1661,7 @@
         <v>8.1813078936337824</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>148</v>
       </c>
@@ -1689,7 +1690,7 @@
         <v>8.4674560537782675</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>148</v>
       </c>
@@ -1718,7 +1719,7 @@
         <v>8.7634099264271512</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>202</v>
       </c>
@@ -1748,7 +1749,7 @@
         <v>86.460524321264955</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>202</v>
       </c>
@@ -1778,7 +1779,7 @@
         <v>87.89444169204053</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>202</v>
       </c>
@@ -1808,7 +1809,7 @@
         <v>89.352140077821005</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>202</v>
       </c>
@@ -1838,7 +1839,7 @@
         <v>90.834013878371721</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>202</v>
       </c>
@@ -1868,7 +1869,7 @@
         <v>92.340464034439464</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>193</v>
       </c>
@@ -1897,7 +1898,7 @@
         <v>97.708742857142852</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>193</v>
       </c>
@@ -1926,7 +1927,7 @@
         <v>98.622035714285715</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>193</v>
       </c>
@@ -1955,7 +1956,7 @@
         <v>98.785214285714289</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>193</v>
       </c>
@@ -1984,7 +1985,7 @@
         <v>98.948392857142849</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>193</v>
       </c>
@@ -2013,7 +2014,7 @@
         <v>99.111571428571423</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>193</v>
       </c>
@@ -2042,7 +2043,7 @@
         <v>99.274749999999997</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>193</v>
       </c>
@@ -2071,7 +2072,7 @@
         <v>99.437928571428571</v>
       </c>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>193</v>
       </c>
@@ -2100,7 +2101,7 @@
         <v>99.601107142857131</v>
       </c>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>193</v>
       </c>
@@ -2129,7 +2130,7 @@
         <v>99.764285714285705</v>
       </c>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>193</v>
       </c>
@@ -2158,7 +2159,7 @@
         <v>99.927464285714279</v>
       </c>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>200</v>
       </c>
@@ -2187,7 +2188,7 @@
         <v>90.92222000000001</v>
       </c>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>200</v>
       </c>
@@ -2216,7 +2217,7 @@
         <v>91.911683266000011</v>
       </c>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>200</v>
       </c>
@@ -2245,7 +2246,7 @@
         <v>92.91184357532002</v>
       </c>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>200</v>
       </c>
@@ -2274,7 +2275,7 @@
         <v>93.922815922499808</v>
       </c>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>200</v>
       </c>
@@ -2303,7 +2304,7 @@
         <v>94.944716532265687</v>
       </c>
     </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>203</v>
       </c>
@@ -2332,7 +2333,7 @@
         <v>361906.34571078792</v>
       </c>
     </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>203</v>
       </c>
@@ -2361,7 +2362,7 @@
         <v>387019.50024189468</v>
       </c>
     </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>203</v>
       </c>
@@ -2390,7 +2391,7 @@
         <v>412231.55552550871</v>
       </c>
     </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>203</v>
       </c>
@@ -2419,7 +2420,7 @@
         <v>437542.51156162989</v>
       </c>
     </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>203</v>
       </c>
@@ -2448,7 +2449,7 @@
         <v>462952.36835025827</v>
       </c>
     </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>203</v>
       </c>
@@ -2477,7 +2478,7 @@
         <v>344656.92064585851</v>
       </c>
     </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>203</v>
       </c>
@@ -2506,7 +2507,7 @@
         <v>364402.73401411739</v>
       </c>
     </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>203</v>
       </c>
@@ -2535,7 +2536,7 @@
         <v>384225.81483198522</v>
       </c>
     </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>203</v>
       </c>
@@ -2564,7 +2565,7 @@
         <v>404126.16309946158</v>
       </c>
     </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>203</v>
       </c>
@@ -2593,7 +2594,7 @@
         <v>424103.77881654678</v>
       </c>
     </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>204</v>
       </c>
@@ -2622,7 +2623,7 @@
         <v>158761.89014095199</v>
       </c>
     </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>204</v>
       </c>
@@ -2651,7 +2652,7 @@
         <v>164342.37057940639</v>
       </c>
     </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>204</v>
       </c>
@@ -2680,7 +2681,7 @@
         <v>170114.7941430413</v>
       </c>
     </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>204</v>
       </c>
@@ -2709,7 +2710,7 @@
         <v>176085.65498697289</v>
       </c>
     </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>204</v>
       </c>
@@ -2738,7 +2739,7 @@
         <v>182261.6641668115</v>
       </c>
     </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>205</v>
       </c>
@@ -2767,7 +2768,7 @@
         <v>7026</v>
       </c>
     </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>205</v>
       </c>
@@ -2796,7 +2797,7 @@
         <v>7500.1430549519973</v>
       </c>
     </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>205</v>
       </c>
@@ -2825,7 +2826,7 @@
         <v>7861.0280628179989</v>
       </c>
     </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>205</v>
       </c>
@@ -2854,7 +2855,7 @@
         <v>8225.1167425979966</v>
       </c>
     </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>205</v>
       </c>
@@ -2883,7 +2884,7 @@
         <v>8592.4090942919956</v>
       </c>
     </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>207</v>
       </c>
@@ -2912,7 +2913,7 @@
         <v>272575.96766625863</v>
       </c>
     </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>207</v>
       </c>
@@ -2941,7 +2942,7 @@
         <v>287876.12222860788</v>
       </c>
     </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>207</v>
       </c>
@@ -2970,7 +2971,7 @@
         <v>304033.49472771061</v>
       </c>
     </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>207</v>
       </c>
@@ -2999,7 +3000,7 @@
         <v>321096.01419443771</v>
       </c>
     </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>207</v>
       </c>
@@ -3028,7 +3029,7 @@
         <v>339114.28347773122</v>
       </c>
     </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>228</v>
       </c>
@@ -3057,7 +3058,7 @@
         <v>892.42950861146085</v>
       </c>
     </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A83">
         <v>228</v>
       </c>
@@ -3086,7 +3087,7 @@
         <v>1019.5881230993029</v>
       </c>
     </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>228</v>
       </c>
@@ -3115,7 +3116,7 @@
         <v>1147.967597954756</v>
       </c>
     </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>228</v>
       </c>
@@ -3144,7 +3145,7 @@
         <v>1277.5679331778181</v>
       </c>
     </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>228</v>
       </c>
@@ -3173,7 +3174,7 @@
         <v>1408.3891287684901</v>
       </c>
     </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>228</v>
       </c>
@@ -3202,7 +3203,7 @@
         <v>796.70494376731313</v>
       </c>
     </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>228</v>
       </c>
@@ -3231,7 +3232,7 @@
         <v>917.28571818365663</v>
       </c>
     </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>228</v>
       </c>
@@ -3260,7 +3261,7 @@
         <v>1055.298221956233</v>
       </c>
     </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>228</v>
       </c>
@@ -3289,7 +3290,7 @@
         <v>1210.984111882826</v>
       </c>
     </row>
-    <row r="91" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A91">
         <v>228</v>
       </c>
@@ -3318,7 +3319,7 @@
         <v>1384.585044761219</v>
       </c>
     </row>
-    <row r="92" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A92">
         <v>244</v>
       </c>
@@ -3347,7 +3348,7 @@
         <v>19.733333333333331</v>
       </c>
     </row>
-    <row r="93" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A93">
         <v>244</v>
       </c>
@@ -3376,7 +3377,7 @@
         <v>19.196888888888889</v>
       </c>
     </row>
-    <row r="94" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>244</v>
       </c>
@@ -3405,7 +3406,7 @@
         <v>18.66577777777778</v>
       </c>
     </row>
-    <row r="95" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A95">
         <v>244</v>
       </c>
@@ -3434,7 +3435,7 @@
         <v>18.14</v>
       </c>
     </row>
-    <row r="96" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A96">
         <v>244</v>
       </c>
@@ -3463,7 +3464,7 @@
         <v>17.61955555555555</v>
       </c>
     </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A97">
         <v>245</v>
       </c>
@@ -3492,7 +3493,7 @@
         <v>89.198827494123194</v>
       </c>
     </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A98">
         <v>245</v>
       </c>
@@ -3521,7 +3522,7 @@
         <v>89.380807536188684</v>
       </c>
     </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>245</v>
       </c>
@@ -3550,7 +3551,7 @@
         <v>89.563090584620838</v>
       </c>
     </row>
-    <row r="100" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A100">
         <v>245</v>
       </c>
@@ -3579,7 +3580,7 @@
         <v>89.745677098501574</v>
       </c>
     </row>
-    <row r="101" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A101">
         <v>245</v>
       </c>
@@ -3608,7 +3609,7 @@
         <v>89.928567537571354</v>
       </c>
     </row>
-    <row r="102" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A102">
         <v>245</v>
       </c>
@@ -3637,7 +3638,7 @@
         <v>90.11176236223001</v>
       </c>
     </row>
-    <row r="103" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A103">
         <v>245</v>
       </c>
@@ -3666,7 +3667,7 @@
         <v>90.295262033537696</v>
       </c>
     </row>
-    <row r="104" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A104">
         <v>245</v>
       </c>
@@ -3695,7 +3696,7 @@
         <v>90.479067013215754</v>
       </c>
     </row>
-    <row r="105" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A105">
         <v>245</v>
       </c>
@@ -3724,7 +3725,7 @@
         <v>90.663177763647781</v>
       </c>
     </row>
-    <row r="106" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A106">
         <v>245</v>
       </c>
@@ -3753,7 +3754,7 @@
         <v>90.847594747880279</v>
       </c>
     </row>
-    <row r="107" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A107">
         <v>245</v>
       </c>
@@ -3782,7 +3783,7 @@
         <v>89.125900000000001</v>
       </c>
     </row>
-    <row r="108" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A108">
         <v>245</v>
       </c>
@@ -3811,7 +3812,7 @@
         <v>89.909943499999997</v>
       </c>
     </row>
-    <row r="109" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A109">
         <v>245</v>
       </c>
@@ -3840,7 +3841,7 @@
         <v>90.695220000000006</v>
       </c>
     </row>
-    <row r="110" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A110">
         <v>245</v>
       </c>
@@ -3869,7 +3870,7 @@
         <v>91.481729500000014</v>
       </c>
     </row>
-    <row r="111" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A111">
         <v>245</v>
       </c>
@@ -3898,7 +3899,7 @@
         <v>92.269472000000007</v>
       </c>
     </row>
-    <row r="112" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A112">
         <v>245</v>
       </c>
@@ -3927,7 +3928,7 @@
         <v>93.058447500000014</v>
       </c>
     </row>
-    <row r="113" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A113">
         <v>245</v>
       </c>
@@ -3956,7 +3957,7 @@
         <v>93.84865600000002</v>
       </c>
     </row>
-    <row r="114" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A114">
         <v>245</v>
       </c>
@@ -3985,7 +3986,7 @@
         <v>94.640097500000024</v>
       </c>
     </row>
-    <row r="115" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A115">
         <v>245</v>
       </c>
@@ -4014,7 +4015,7 @@
         <v>95.432772000000014</v>
       </c>
     </row>
-    <row r="116" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A116">
         <v>245</v>
       </c>
@@ -4043,7 +4044,7 @@
         <v>96.226679500000017</v>
       </c>
     </row>
-    <row r="117" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A117">
         <v>276</v>
       </c>
@@ -4072,7 +4073,7 @@
         <v>64.626946951668998</v>
       </c>
     </row>
-    <row r="118" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A118">
         <v>276</v>
       </c>
@@ -4101,7 +4102,7 @@
         <v>61.797659797529029</v>
       </c>
     </row>
-    <row r="119" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A119">
         <v>276</v>
       </c>
@@ -4130,7 +4131,7 @@
         <v>58.996085245839843</v>
       </c>
     </row>
-    <row r="120" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A120">
         <v>276</v>
       </c>
@@ -4159,7 +4160,7 @@
         <v>56.222223296601427</v>
       </c>
     </row>
-    <row r="121" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A121">
         <v>276</v>
       </c>
@@ -4188,7 +4189,7 @@
         <v>53.476073949813816</v>
       </c>
     </row>
-    <row r="122" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A122">
         <v>276</v>
       </c>
@@ -4217,7 +4218,7 @@
         <v>50.757637205477003</v>
       </c>
     </row>
-    <row r="123" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A123">
         <v>276</v>
       </c>
@@ -4246,7 +4247,7 @@
         <v>48.06691306359096</v>
       </c>
     </row>
-    <row r="124" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A124">
         <v>276</v>
       </c>
@@ -4275,7 +4276,7 @@
         <v>45.403901524155707</v>
       </c>
     </row>
-    <row r="125" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A125">
         <v>276</v>
       </c>
@@ -4304,7 +4305,7 @@
         <v>42.768602587171237</v>
       </c>
     </row>
-    <row r="126" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A126">
         <v>276</v>
       </c>
@@ -4333,7 +4334,7 @@
         <v>40.16101625263758</v>
       </c>
     </row>
-    <row r="127" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A127">
         <v>276</v>
       </c>
@@ -4362,7 +4363,7 @@
         <v>69.3338001487799</v>
       </c>
     </row>
-    <row r="128" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A128">
         <v>276</v>
       </c>
@@ -4391,7 +4392,7 @@
         <v>67.352972385300021</v>
       </c>
     </row>
-    <row r="129" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A129">
         <v>276</v>
       </c>
@@ -4420,7 +4421,7 @@
         <v>65.426674283148913</v>
       </c>
     </row>
-    <row r="130" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A130">
         <v>276</v>
       </c>
@@ -4449,7 +4450,7 @@
         <v>63.553443269459287</v>
       </c>
     </row>
-    <row r="131" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A131">
         <v>276</v>
       </c>
@@ -4478,7 +4479,7 @@
         <v>61.731855251410558</v>
       </c>
     </row>
-    <row r="132" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A132">
         <v>276</v>
       </c>
@@ -4507,7 +4508,7 @@
         <v>59.960523618738179</v>
       </c>
     </row>
-    <row r="133" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A133">
         <v>276</v>
       </c>
@@ -4536,7 +4537,7 @@
         <v>58.238098271797057</v>
       </c>
     </row>
-    <row r="134" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A134">
         <v>276</v>
       </c>
@@ -4565,7 +4566,7 @@
         <v>56.563264674531062</v>
       </c>
     </row>
-    <row r="135" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A135">
         <v>276</v>
       </c>
@@ -4594,7 +4595,7 @@
         <v>54.934742931716322</v>
       </c>
     </row>
-    <row r="136" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A136">
         <v>276</v>
       </c>
@@ -4623,7 +4624,7 @@
         <v>53.351286889862124</v>
       </c>
     </row>
-    <row r="137" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A137">
         <v>277</v>
       </c>
@@ -4651,8 +4652,16 @@
       <c r="I137">
         <v>65.423590000000004</v>
       </c>
-    </row>
-    <row r="138" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J137">
+        <f>+G137*0.95</f>
+        <v>64.074650000000005</v>
+      </c>
+      <c r="K137">
+        <f>+G137*1.05</f>
+        <v>70.81935</v>
+      </c>
+    </row>
+    <row r="138" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A138">
         <v>277</v>
       </c>
@@ -4680,8 +4689,16 @@
       <c r="I138">
         <v>63.790038399999993</v>
       </c>
-    </row>
-    <row r="139" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J138">
+        <f t="shared" ref="J138:J146" si="1">+G138*0.95</f>
+        <v>62.532799999999995</v>
+      </c>
+      <c r="K138">
+        <f t="shared" ref="K138:K146" si="2">+G138*1.05</f>
+        <v>69.115200000000002</v>
+      </c>
+    </row>
+    <row r="139" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A139">
         <v>277</v>
       </c>
@@ -4709,8 +4726,16 @@
       <c r="I139">
         <v>62.159408199999987</v>
       </c>
-    </row>
-    <row r="140" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J139">
+        <f t="shared" si="1"/>
+        <v>60.990949999999991</v>
+      </c>
+      <c r="K139">
+        <f t="shared" si="2"/>
+        <v>67.411050000000003</v>
+      </c>
+    </row>
+    <row r="140" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A140">
         <v>277</v>
       </c>
@@ -4738,8 +4763,16 @@
       <c r="I140">
         <v>60.531699400000001</v>
       </c>
-    </row>
-    <row r="141" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J140">
+        <f t="shared" si="1"/>
+        <v>59.449100000000001</v>
+      </c>
+      <c r="K140">
+        <f t="shared" si="2"/>
+        <v>65.706900000000005</v>
+      </c>
+    </row>
+    <row r="141" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A141">
         <v>277</v>
       </c>
@@ -4767,8 +4800,16 @@
       <c r="I141">
         <v>58.906911999999991</v>
       </c>
-    </row>
-    <row r="142" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J141">
+        <f t="shared" si="1"/>
+        <v>57.907249999999998</v>
+      </c>
+      <c r="K141">
+        <f t="shared" si="2"/>
+        <v>64.002750000000006</v>
+      </c>
+    </row>
+    <row r="142" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A142">
         <v>277</v>
       </c>
@@ -4796,8 +4837,16 @@
       <c r="I142">
         <v>57.285045999999987</v>
       </c>
-    </row>
-    <row r="143" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J142">
+        <f t="shared" si="1"/>
+        <v>56.365399999999987</v>
+      </c>
+      <c r="K142">
+        <f t="shared" si="2"/>
+        <v>62.298599999999986</v>
+      </c>
+    </row>
+    <row r="143" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A143">
         <v>277</v>
       </c>
@@ -4825,8 +4874,16 @@
       <c r="I143">
         <v>55.666101400000002</v>
       </c>
-    </row>
-    <row r="144" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J143">
+        <f t="shared" si="1"/>
+        <v>54.823549999999997</v>
+      </c>
+      <c r="K143">
+        <f t="shared" si="2"/>
+        <v>60.594450000000009</v>
+      </c>
+    </row>
+    <row r="144" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A144">
         <v>277</v>
       </c>
@@ -4854,8 +4911,16 @@
       <c r="I144">
         <v>54.050078199999987</v>
       </c>
-    </row>
-    <row r="145" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J144">
+        <f t="shared" si="1"/>
+        <v>53.281699999999987</v>
+      </c>
+      <c r="K144">
+        <f t="shared" si="2"/>
+        <v>58.890299999999996</v>
+      </c>
+    </row>
+    <row r="145" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A145">
         <v>277</v>
       </c>
@@ -4883,8 +4948,16 @@
       <c r="I145">
         <v>52.436976399999992</v>
       </c>
-    </row>
-    <row r="146" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J145">
+        <f t="shared" si="1"/>
+        <v>51.739849999999983</v>
+      </c>
+      <c r="K145">
+        <f t="shared" si="2"/>
+        <v>57.186149999999991</v>
+      </c>
+    </row>
+    <row r="146" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A146">
         <v>277</v>
       </c>
@@ -4912,8 +4985,16 @@
       <c r="I146">
         <v>50.826795999999987</v>
       </c>
-    </row>
-    <row r="147" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J146">
+        <f t="shared" si="1"/>
+        <v>50.197999999999986</v>
+      </c>
+      <c r="K146">
+        <f t="shared" si="2"/>
+        <v>55.481999999999992</v>
+      </c>
+    </row>
+    <row r="147" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A147">
         <v>277</v>
       </c>
@@ -4941,8 +5022,16 @@
       <c r="I147">
         <v>65.851630338904542</v>
       </c>
-    </row>
-    <row r="148" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J147">
+        <f>+G147*0.95</f>
+        <v>64.493864764906505</v>
+      </c>
+      <c r="K147">
+        <f>+G147*1.05</f>
+        <v>71.282692634896677</v>
+      </c>
+    </row>
+    <row r="148" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A148">
         <v>277</v>
       </c>
@@ -4970,8 +5059,16 @@
       <c r="I148">
         <v>64.366708412510363</v>
       </c>
-    </row>
-    <row r="149" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J148">
+        <f t="shared" ref="J148:J156" si="3">+G148*0.95</f>
+        <v>63.098104418413833</v>
+      </c>
+      <c r="K148">
+        <f t="shared" ref="K148:K156" si="4">+G148*1.05</f>
+        <v>69.740010146667927</v>
+      </c>
+    </row>
+    <row r="149" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A149">
         <v>277</v>
       </c>
@@ -4999,8 +5096,16 @@
       <c r="I149">
         <v>62.915216483343421</v>
       </c>
-    </row>
-    <row r="150" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J149">
+        <f t="shared" si="3"/>
+        <v>61.732550773782535</v>
+      </c>
+      <c r="K149">
+        <f t="shared" si="4"/>
+        <v>68.230714013128065</v>
+      </c>
+    </row>
+    <row r="150" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A150">
         <v>277</v>
       </c>
@@ -5028,8 +5133,16 @@
       <c r="I150">
         <v>61.496403070076219</v>
       </c>
-    </row>
-    <row r="151" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J150">
+        <f t="shared" si="3"/>
+        <v>60.396550105006106</v>
+      </c>
+      <c r="K150">
+        <f t="shared" si="4"/>
+        <v>66.754081695006761</v>
+      </c>
+    </row>
+    <row r="151" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A151">
         <v>277</v>
       </c>
@@ -5057,8 +5170,16 @@
       <c r="I151">
         <v>60.109533560671402</v>
       </c>
-    </row>
-    <row r="152" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J151">
+        <f t="shared" si="3"/>
+        <v>59.089462833855379</v>
+      </c>
+      <c r="K151">
+        <f t="shared" si="4"/>
+        <v>65.309406290050688</v>
+      </c>
+    </row>
+    <row r="152" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A152">
         <v>277</v>
       </c>
@@ -5086,8 +5207,16 @@
       <c r="I152">
         <v>58.75388983418766</v>
       </c>
-    </row>
-    <row r="153" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J152">
+        <f t="shared" si="3"/>
+        <v>57.810663223695791</v>
+      </c>
+      <c r="K152">
+        <f t="shared" si="4"/>
+        <v>63.895996194611136</v>
+      </c>
+    </row>
+    <row r="153" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A153">
         <v>277</v>
       </c>
@@ -5115,8 +5244,16 @@
       <c r="I153">
         <v>57.428769891054131</v>
       </c>
-    </row>
-    <row r="154" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J153">
+        <f t="shared" si="3"/>
+        <v>56.559539079930978</v>
+      </c>
+      <c r="K153">
+        <f t="shared" si="4"/>
+        <v>62.513174772555296</v>
+      </c>
+    </row>
+    <row r="154" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A154">
         <v>277</v>
       </c>
@@ -5144,8 +5281,16 @@
       <c r="I154">
         <v>56.133487491624052</v>
       </c>
-    </row>
-    <row r="155" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J154">
+        <f t="shared" si="3"/>
+        <v>55.335491456929368</v>
+      </c>
+      <c r="K154">
+        <f t="shared" si="4"/>
+        <v>61.160280031342985</v>
+      </c>
+    </row>
+    <row r="155" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A155">
         <v>277</v>
       </c>
@@ -5173,8 +5318,16 @@
       <c r="I155">
         <v>54.867371802822348</v>
       </c>
-    </row>
-    <row r="156" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J155">
+        <f t="shared" si="3"/>
+        <v>54.137934371293333</v>
+      </c>
+      <c r="K155">
+        <f t="shared" si="4"/>
+        <v>59.836664305113693</v>
+      </c>
+    </row>
+    <row r="156" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A156">
         <v>277</v>
       </c>
@@ -5202,8 +5355,16 @@
       <c r="I156">
         <v>53.629767052706171</v>
       </c>
-    </row>
-    <row r="157" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J156">
+        <f t="shared" si="3"/>
+        <v>52.966294521333673</v>
+      </c>
+      <c r="K156">
+        <f t="shared" si="4"/>
+        <v>58.541693944631952</v>
+      </c>
+    </row>
+    <row r="157" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A157">
         <v>325</v>
       </c>
@@ -5232,7 +5393,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="158" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A158">
         <v>325</v>
       </c>
@@ -5261,7 +5422,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="159" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A159">
         <v>325</v>
       </c>
@@ -5290,7 +5451,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="160" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A160">
         <v>325</v>
       </c>
@@ -5319,7 +5480,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="161" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A161">
         <v>325</v>
       </c>
@@ -5348,7 +5509,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="162" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A162">
         <v>332</v>
       </c>
@@ -5377,7 +5538,7 @@
         <v>0.64546314585089737</v>
       </c>
     </row>
-    <row r="163" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A163">
         <v>332</v>
       </c>
@@ -5406,7 +5567,7 @@
         <v>0.51469902830302305</v>
       </c>
     </row>
-    <row r="164" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A164">
         <v>332</v>
       </c>
@@ -5435,7 +5596,7 @@
         <v>0.41042203194026261</v>
       </c>
     </row>
-    <row r="165" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A165">
         <v>332</v>
       </c>
@@ -5464,7 +5625,7 @@
         <v>0.32726787299048538</v>
       </c>
     </row>
-    <row r="166" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A166">
         <v>332</v>
       </c>
@@ -5493,7 +5654,7 @@
         <v>0.26095849634300861</v>
       </c>
     </row>
-    <row r="167" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A167">
         <v>332</v>
       </c>
@@ -5522,7 +5683,7 @@
         <v>0.65439130434782633</v>
       </c>
     </row>
-    <row r="168" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A168">
         <v>332</v>
       </c>
@@ -5551,7 +5712,7 @@
         <v>0.52181843478260892</v>
       </c>
     </row>
-    <row r="169" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A169">
         <v>332</v>
       </c>
@@ -5580,7 +5741,7 @@
         <v>0.41609906086956538</v>
       </c>
     </row>
-    <row r="170" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A170">
         <v>332</v>
       </c>
@@ -5609,7 +5770,7 @@
         <v>0.33179469913043491</v>
       </c>
     </row>
-    <row r="171" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A171">
         <v>332</v>
       </c>
@@ -5638,7 +5799,7 @@
         <v>0.26456811965217403</v>
       </c>
     </row>
-    <row r="172" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A172">
         <v>334</v>
       </c>
@@ -5667,7 +5828,7 @@
         <v>93.70400000673547</v>
       </c>
     </row>
-    <row r="173" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A173">
         <v>334</v>
       </c>
@@ -5696,7 +5857,7 @@
         <v>94.782871493406859</v>
       </c>
     </row>
-    <row r="174" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A174">
         <v>334</v>
       </c>
@@ -5725,7 +5886,7 @@
         <v>95.863802289969655</v>
       </c>
     </row>
-    <row r="175" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A175">
         <v>334</v>
       </c>
@@ -5754,7 +5915,7 @@
         <v>96.946792396423888</v>
       </c>
     </row>
-    <row r="176" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A176">
         <v>334</v>
       </c>
@@ -5783,7 +5944,7 @@
         <v>98.0318418127695</v>
       </c>
     </row>
-    <row r="177" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A177">
         <v>334</v>
       </c>
@@ -5812,7 +5973,7 @@
         <v>92.93801595829882</v>
       </c>
     </row>
-    <row r="178" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A178">
         <v>334</v>
       </c>
@@ -5841,7 +6002,7 @@
         <v>93.968919736860101</v>
       </c>
     </row>
-    <row r="179" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A179">
         <v>334</v>
       </c>
@@ -5870,7 +6031,7 @@
         <v>95.131696762608669</v>
       </c>
     </row>
-    <row r="180" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A180">
         <v>334</v>
       </c>
@@ -5899,7 +6060,7 @@
         <v>96.426755945691355</v>
       </c>
     </row>
-    <row r="181" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A181">
         <v>334</v>
       </c>
@@ -5928,7 +6089,7 @@
         <v>97.854506196255059</v>
       </c>
     </row>
-    <row r="182" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A182">
         <v>361</v>
       </c>
@@ -5957,7 +6118,7 @@
         <v>4.83446</v>
       </c>
     </row>
-    <row r="183" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A183">
         <v>361</v>
       </c>
@@ -5986,7 +6147,7 @@
         <v>4.8645499999999995</v>
       </c>
     </row>
-    <row r="184" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A184">
         <v>361</v>
       </c>
@@ -6015,7 +6176,7 @@
         <v>4.8846099999999995</v>
       </c>
     </row>
-    <row r="185" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A185">
         <v>361</v>
       </c>
@@ -6044,7 +6205,7 @@
         <v>4.9247299999999994</v>
       </c>
     </row>
-    <row r="186" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A186">
         <v>361</v>
       </c>
@@ -6073,7 +6234,7 @@
         <v>4.9748799999999997</v>
       </c>
     </row>
-    <row r="187" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A187" s="3">
         <v>364</v>
       </c>
@@ -6102,7 +6263,7 @@
         <v>115494.72</v>
       </c>
     </row>
-    <row r="188" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A188" s="3">
         <v>364</v>
       </c>
@@ -6131,7 +6292,7 @@
         <v>126091.36056</v>
       </c>
     </row>
-    <row r="189" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A189" s="3">
         <v>364</v>
       </c>
@@ -6160,7 +6321,7 @@
         <v>137652.38203200011</v>
       </c>
     </row>
-    <row r="190" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A190" s="3">
         <v>364</v>
       </c>
@@ -6189,7 +6350,7 @@
         <v>150264.6941928</v>
       </c>
     </row>
-    <row r="191" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A191" s="3">
         <v>364</v>
       </c>
@@ -6218,7 +6379,7 @@
         <v>164022.94496544011</v>
       </c>
     </row>
-    <row r="192" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A192" s="3">
         <v>367</v>
       </c>
@@ -6247,7 +6408,7 @@
         <v>5.5479450746268659</v>
       </c>
     </row>
-    <row r="193" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A193" s="3">
         <v>367</v>
       </c>
@@ -6276,7 +6437,7 @@
         <v>5.6197363811343282</v>
       </c>
     </row>
-    <row r="194" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A194" s="3">
         <v>367</v>
       </c>
@@ -6305,7 +6466,7 @@
         <v>5.6924087192644777</v>
       </c>
     </row>
-    <row r="195" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A195" s="3">
         <v>367</v>
       </c>
@@ -6334,7 +6495,7 @@
         <v>5.7659725305191172</v>
       </c>
     </row>
-    <row r="196" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A196" s="3">
         <v>367</v>
       </c>
@@ -6363,7 +6524,7 @@
         <v>5.8404383771269233</v>
       </c>
     </row>
-    <row r="197" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A197" s="3">
         <v>369</v>
       </c>
@@ -6392,7 +6553,7 @@
         <v>88.128</v>
       </c>
     </row>
-    <row r="198" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A198" s="3">
         <v>369</v>
       </c>
@@ -6421,7 +6582,7 @@
         <v>90.340012799999997</v>
       </c>
     </row>
-    <row r="199" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A199" s="3">
         <v>369</v>
       </c>
@@ -6450,7 +6611,7 @@
         <v>92.605254912000021</v>
       </c>
     </row>
-    <row r="200" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A200" s="3">
         <v>369</v>
       </c>
@@ -6479,7 +6640,7 @@
         <v>94.924970703359989</v>
       </c>
     </row>
-    <row r="201" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A201" s="3">
         <v>369</v>
       </c>
@@ -6508,7 +6669,7 @@
         <v>97.3004330244096</v>
       </c>
     </row>
-    <row r="202" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A202" s="3">
         <v>377</v>
       </c>
@@ -6537,7 +6698,7 @@
         <v>14193.63602034</v>
       </c>
     </row>
-    <row r="203" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A203" s="3">
         <v>377</v>
       </c>
@@ -6566,7 +6727,7 @@
         <v>16404.294830507952</v>
       </c>
     </row>
-    <row r="204" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A204" s="3">
         <v>377</v>
       </c>
@@ -6595,7 +6756,7 @@
         <v>18958.794473268641</v>
       </c>
     </row>
-    <row r="205" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A205" s="3">
         <v>377</v>
       </c>
@@ -6624,7 +6785,7 @@
         <v>21910.547375171111</v>
       </c>
     </row>
-    <row r="206" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A206" s="3">
         <v>377</v>
       </c>
@@ -6653,7 +6814,7 @@
         <v>25321.253271995771</v>
       </c>
     </row>
-    <row r="207" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A207">
         <v>424</v>
       </c>
@@ -6682,7 +6843,7 @@
         <v>12.5</v>
       </c>
     </row>
-    <row r="208" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A208">
         <v>424</v>
       </c>
@@ -6711,7 +6872,7 @@
         <v>13.2</v>
       </c>
     </row>
-    <row r="209" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A209">
         <v>424</v>
       </c>
@@ -6740,7 +6901,7 @@
         <v>13.8</v>
       </c>
     </row>
-    <row r="210" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A210">
         <v>424</v>
       </c>
@@ -6769,7 +6930,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="211" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A211">
         <v>424</v>
       </c>
@@ -6798,7 +6959,7 @@
         <v>14.5</v>
       </c>
     </row>
-    <row r="212" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A212">
         <v>460</v>
       </c>
@@ -6827,7 +6988,7 @@
         <v>95.125032000000004</v>
       </c>
     </row>
-    <row r="213" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A213">
         <v>460</v>
       </c>
@@ -6856,7 +7017,7 @@
         <v>96.160232469600004</v>
       </c>
     </row>
-    <row r="214" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A214">
         <v>460</v>
       </c>
@@ -6885,7 +7046,7 @@
         <v>97.206624445392023</v>
       </c>
     </row>
-    <row r="215" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A215">
         <v>460</v>
       </c>
@@ -6914,7 +7075,7 @@
         <v>98.545849202319999</v>
       </c>
     </row>
-    <row r="216" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A216">
         <v>460</v>
       </c>
@@ -6943,7 +7104,7 @@
         <v>98.831307694343209</v>
       </c>
     </row>
-    <row r="217" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A217">
         <v>77</v>
       </c>
@@ -6972,7 +7133,7 @@
         <v>98.67895</v>
       </c>
     </row>
-    <row r="218" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A218">
         <v>77</v>
       </c>
@@ -7001,7 +7162,7 @@
         <v>98.965739499999998</v>
       </c>
     </row>
-    <row r="219" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A219">
         <v>77</v>
       </c>
@@ -7030,7 +7191,7 @@
         <v>99.255396895000004</v>
       </c>
     </row>
-    <row r="220" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A220">
         <v>77</v>
       </c>
@@ -7059,7 +7220,7 @@
         <v>99.547950863950007</v>
       </c>
     </row>
-    <row r="221" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A221">
         <v>77</v>
       </c>
@@ -7088,7 +7249,7 @@
         <v>99.843430372589509</v>
       </c>
     </row>
-    <row r="222" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A222">
         <v>98</v>
       </c>
@@ -7117,7 +7278,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="223" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A223">
         <v>98</v>
       </c>
@@ -7146,7 +7307,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="224" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A224">
         <v>98</v>
       </c>
@@ -7175,7 +7336,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="225" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A225">
         <v>98</v>
       </c>
@@ -7204,7 +7365,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="226" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A226">
         <v>98</v>
       </c>
@@ -7233,7 +7394,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="227" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A227" s="3">
         <v>386.1</v>
       </c>
@@ -7262,7 +7423,7 @@
         <v>6025.5908288085884</v>
       </c>
     </row>
-    <row r="228" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A228" s="3">
         <v>386.1</v>
       </c>
@@ -7291,7 +7452,7 @@
         <v>7132.9729466473937</v>
       </c>
     </row>
-    <row r="229" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A229" s="3">
         <v>386.1</v>
       </c>
@@ -7320,7 +7481,7 @@
         <v>8387.9290364164917</v>
       </c>
     </row>
-    <row r="230" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A230" s="3">
         <v>386.1</v>
       </c>
@@ -7349,7 +7510,7 @@
         <v>9792.4915984875806</v>
       </c>
     </row>
-    <row r="231" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A231" s="3">
         <v>386.1</v>
       </c>
@@ -7378,7 +7539,7 @@
         <v>11348.693133232369</v>
       </c>
     </row>
-    <row r="232" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A232" s="3">
         <v>386.2</v>
       </c>
@@ -7407,7 +7568,7 @@
         <v>9176.5019107995558</v>
       </c>
     </row>
-    <row r="233" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A233" s="3">
         <v>386.2</v>
       </c>
@@ -7436,7 +7597,7 @@
         <v>10283.967217993961</v>
       </c>
     </row>
-    <row r="234" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A234" s="3">
         <v>386.2</v>
       </c>
@@ -7465,7 +7626,7 @@
         <v>11524.99750015523</v>
       </c>
     </row>
-    <row r="235" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A235" s="3">
         <v>386.2</v>
       </c>
@@ -7494,7 +7655,7 @@
         <v>12915.691019463869</v>
       </c>
     </row>
-    <row r="236" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A236" s="3">
         <v>386.2</v>
       </c>
@@ -7523,7 +7684,7 @@
         <v>14474.085149544269</v>
       </c>
     </row>
-    <row r="237" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A237" s="3">
         <v>386.3</v>
       </c>
@@ -7552,7 +7713,7 @@
         <v>6775.7920969396118</v>
       </c>
     </row>
-    <row r="238" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A238" s="3">
         <v>386.3</v>
       </c>
@@ -7581,7 +7742,7 @@
         <v>7687.612830857006</v>
       </c>
     </row>
-    <row r="239" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A239" s="3">
         <v>386.3</v>
       </c>
@@ -7610,7 +7771,7 @@
         <v>8759.3798750710612</v>
       </c>
     </row>
-    <row r="240" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A240" s="3">
         <v>386.3</v>
       </c>
@@ -7639,7 +7800,7 @@
         <v>9993.3389311351038</v>
       </c>
     </row>
-    <row r="241" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A241" s="3">
         <v>386.3</v>
       </c>
@@ -7668,7 +7829,7 @@
         <v>11391.73570060247</v>
       </c>
     </row>
-    <row r="242" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A242">
         <v>379</v>
       </c>
@@ -7697,7 +7858,7 @@
         <v>13317.175813442071</v>
       </c>
     </row>
-    <row r="243" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A243">
         <v>274</v>
       </c>
@@ -7726,7 +7887,7 @@
         <v>46054.901058930787</v>
       </c>
     </row>
-    <row r="244" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A244">
         <v>379</v>
       </c>
@@ -7755,7 +7916,7 @@
         <v>13418.021660158851</v>
       </c>
     </row>
-    <row r="245" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A245">
         <v>274</v>
       </c>
@@ -7784,7 +7945,7 @@
         <v>46403.657098334967</v>
       </c>
     </row>
-    <row r="246" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A246">
         <v>379</v>
       </c>
@@ -7813,7 +7974,7 @@
         <v>13536.316299144</v>
       </c>
     </row>
-    <row r="247" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A247">
         <v>274</v>
       </c>
@@ -7842,7 +8003,7 @@
         <v>46812.756442714293</v>
       </c>
     </row>
-    <row r="248" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A248">
         <v>379</v>
       </c>
@@ -7871,7 +8032,7 @@
         <v>13665.23975007113</v>
       </c>
     </row>
-    <row r="249" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A249">
         <v>274</v>
       </c>
@@ -7900,7 +8061,7 @@
         <v>47258.613496777638</v>
       </c>
     </row>
-    <row r="250" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A250">
         <v>379</v>
       </c>
@@ -7929,7 +8090,7 @@
         <v>13801.316029168571</v>
       </c>
     </row>
-    <row r="251" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A251">
         <v>274</v>
       </c>
@@ -7958,7 +8119,7 @@
         <v>47729.20723662855</v>
       </c>
     </row>
-    <row r="252" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A252">
         <v>379</v>
       </c>
@@ -7987,7 +8148,7 @@
         <v>13942.80055708834</v>
       </c>
     </row>
-    <row r="253" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A253">
         <v>274</v>
       </c>
@@ -8016,7 +8177,7 @@
         <v>48218.50436884314</v>
       </c>
     </row>
-    <row r="254" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A254">
         <v>379</v>
       </c>
@@ -8045,7 +8206,7 @@
         <v>14088.84540208515</v>
       </c>
     </row>
-    <row r="255" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A255">
         <v>274</v>
       </c>
@@ -8074,7 +8235,7 @@
         <v>48723.572483938951</v>
       </c>
     </row>
-    <row r="256" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A256">
         <v>379</v>
       </c>
@@ -8103,7 +8264,7 @@
         <v>14239.06717106818</v>
       </c>
     </row>
-    <row r="257" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A257">
         <v>274</v>
       </c>
@@ -8132,7 +8293,7 @@
         <v>49243.085690367268</v>
       </c>
     </row>
-    <row r="258" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A258">
         <v>379</v>
       </c>
@@ -8161,7 +8322,7 @@
         <v>14393.32333139659</v>
       </c>
     </row>
-    <row r="259" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A259">
         <v>274</v>
       </c>
@@ -8190,7 +8351,7 @@
         <v>49776.551066298169</v>
       </c>
     </row>
-    <row r="260" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A260">
         <v>379</v>
       </c>
@@ -8219,7 +8380,7 @@
         <v>14551.59642655029</v>
       </c>
     </row>
-    <row r="261" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A261">
         <v>274</v>
       </c>
@@ -8248,7 +8409,7 @@
         <v>50323.908241701443</v>
       </c>
     </row>
-    <row r="262" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A262">
         <v>14</v>
       </c>
@@ -8277,7 +8438,7 @@
         <v>59371.884262853768</v>
       </c>
     </row>
-    <row r="263" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A263">
         <v>14</v>
       </c>
@@ -8306,7 +8467,7 @@
         <v>59821.484690416968</v>
       </c>
     </row>
-    <row r="264" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A264">
         <v>14</v>
       </c>
@@ -8335,7 +8496,7 @@
         <v>60348.876962857597</v>
       </c>
     </row>
-    <row r="265" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A265">
         <v>14</v>
       </c>
@@ -8364,7 +8525,7 @@
         <v>60923.655603197178</v>
       </c>
     </row>
-    <row r="266" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A266">
         <v>14</v>
       </c>
@@ -8393,7 +8554,7 @@
         <v>61530.323654041553</v>
       </c>
     </row>
-    <row r="267" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A267">
         <v>14</v>
       </c>
@@ -8422,7 +8583,7 @@
         <v>62161.103267851133</v>
       </c>
     </row>
-    <row r="268" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A268">
         <v>14</v>
       </c>
@@ -8451,7 +8612,7 @@
         <v>62812.214115662013</v>
       </c>
     </row>
-    <row r="269" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A269">
         <v>14</v>
       </c>
@@ -8480,7 +8641,7 @@
         <v>63481.946918379748</v>
       </c>
     </row>
-    <row r="270" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A270">
         <v>14</v>
       </c>
@@ -8509,7 +8670,7 @@
         <v>64169.666223595093</v>
       </c>
     </row>
-    <row r="271" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A271">
         <v>14</v>
       </c>
@@ -8538,7 +8699,7 @@
         <v>64875.294205010192</v>
       </c>
     </row>
-    <row r="272" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A272">
         <v>14</v>
       </c>
@@ -8567,7 +8728,7 @@
         <v>60802.946712188583</v>
       </c>
     </row>
-    <row r="273" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A273">
         <v>14</v>
       </c>
@@ -8596,7 +8757,7 @@
         <v>61412.55539447139</v>
       </c>
     </row>
-    <row r="274" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A274">
         <v>14</v>
       </c>
@@ -8625,7 +8786,7 @@
         <v>62023.951131092377</v>
       </c>
     </row>
-    <row r="275" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A275">
         <v>14</v>
       </c>
@@ -8654,7 +8815,7 @@
         <v>62637.133922051551</v>
       </c>
     </row>
-    <row r="276" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A276">
         <v>14</v>
       </c>
@@ -8683,7 +8844,7 @@
         <v>63252.103767348883</v>
       </c>
     </row>
-    <row r="277" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A277">
         <v>14</v>
       </c>
@@ -8712,7 +8873,7 @@
         <v>63868.860666984387</v>
       </c>
     </row>
-    <row r="278" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A278">
         <v>14</v>
       </c>
@@ -8741,7 +8902,7 @@
         <v>64487.404620958077</v>
       </c>
     </row>
-    <row r="279" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A279">
         <v>14</v>
       </c>
@@ -8770,7 +8931,7 @@
         <v>65107.735629269962</v>
       </c>
     </row>
-    <row r="280" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A280">
         <v>14</v>
       </c>
@@ -8799,7 +8960,7 @@
         <v>65729.853691919998</v>
       </c>
     </row>
-    <row r="281" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A281">
         <v>14</v>
       </c>
@@ -8828,7 +8989,7 @@
         <v>66353.758808908198</v>
       </c>
     </row>
-    <row r="282" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A282">
         <v>379</v>
       </c>
@@ -8857,7 +9018,7 @@
         <v>13638.16461941349</v>
       </c>
     </row>
-    <row r="283" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A283">
         <v>274</v>
       </c>
@@ -8886,7 +9047,7 @@
         <v>47164.979344832544</v>
       </c>
     </row>
-    <row r="284" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A284">
         <v>379</v>
       </c>
@@ -8915,7 +9076,7 @@
         <v>13774.90048522195</v>
       </c>
     </row>
-    <row r="285" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A285">
         <v>274</v>
       </c>
@@ -8944,7 +9105,7 @@
         <v>47637.854138950643</v>
       </c>
     </row>
-    <row r="286" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A286">
         <v>379</v>
       </c>
@@ -8973,7 +9134,7 @@
         <v>13912.037189189839</v>
       </c>
     </row>
-    <row r="287" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A287">
         <v>274</v>
       </c>
@@ -9002,7 +9163,7 @@
         <v>48112.115155044899</v>
       </c>
     </row>
-    <row r="288" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A288">
         <v>379</v>
       </c>
@@ -9031,7 +9192,7 @@
         <v>14049.574731317151</v>
       </c>
     </row>
-    <row r="289" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A289">
         <v>274</v>
       </c>
@@ -9060,7 +9221,7 @@
         <v>48587.762393115328</v>
       </c>
     </row>
-    <row r="290" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A290">
         <v>379</v>
       </c>
@@ -9089,7 +9250,7 @@
         <v>14187.513111603899</v>
       </c>
     </row>
-    <row r="291" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="291" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A291">
         <v>274</v>
       </c>
@@ -9118,7 +9279,7 @@
         <v>49064.795853161922</v>
       </c>
     </row>
-    <row r="292" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A292">
         <v>379</v>
       </c>
@@ -9147,7 +9308,7 @@
         <v>14325.85233005006</v>
       </c>
     </row>
-    <row r="293" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="293" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A293">
         <v>274</v>
       </c>
@@ -9176,7 +9337,7 @@
         <v>49543.215535184667</v>
       </c>
     </row>
-    <row r="294" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A294">
         <v>379</v>
       </c>
@@ -9205,7 +9366,7 @@
         <v>14464.59238665566</v>
       </c>
     </row>
-    <row r="295" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A295">
         <v>274</v>
       </c>
@@ -9234,7 +9395,7 @@
         <v>50023.021439183598</v>
       </c>
     </row>
-    <row r="296" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A296">
         <v>379</v>
       </c>
@@ -9263,7 +9424,7 @@
         <v>14603.73328142068</v>
       </c>
     </row>
-    <row r="297" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A297">
         <v>274</v>
       </c>
@@ -9292,7 +9453,7 @@
         <v>50504.213565158687</v>
       </c>
     </row>
-    <row r="298" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A298">
         <v>379</v>
       </c>
@@ -9321,7 +9482,7 @@
         <v>14743.275014345139</v>
       </c>
     </row>
-    <row r="299" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A299">
         <v>274</v>
       </c>
@@ -9350,7 +9511,7 @@
         <v>50986.791913109962</v>
       </c>
     </row>
-    <row r="300" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A300">
         <v>379</v>
       </c>
@@ -9379,7 +9540,7 @@
         <v>14883.217585429011</v>
       </c>
     </row>
-    <row r="301" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A301">
         <v>274</v>
       </c>
@@ -9408,7 +9569,7 @@
         <v>51470.756483037367</v>
       </c>
     </row>
-    <row r="302" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A302">
         <v>14.1</v>
       </c>
@@ -9437,7 +9598,7 @@
         <v>9487.176818882821</v>
       </c>
     </row>
-    <row r="303" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A303">
         <v>14.2</v>
       </c>
@@ -9466,7 +9627,7 @@
         <v>51315.769893305762</v>
       </c>
     </row>
-    <row r="304" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A304">
         <v>14.1</v>
       </c>
@@ -9495,7 +9656,7 @@
         <v>9582.2949944297943</v>
       </c>
     </row>
-    <row r="305" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A305">
         <v>14.2</v>
       </c>
@@ -9524,7 +9685,7 @@
         <v>51830.260400041603</v>
       </c>
     </row>
-    <row r="306" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A306">
         <v>14.1</v>
       </c>
@@ -9553,7 +9714,7 @@
         <v>9677.6920067997835</v>
       </c>
     </row>
-    <row r="307" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A307">
         <v>14.2</v>
       </c>
@@ -9582,7 +9743,7 @@
         <v>52346.259124292606</v>
       </c>
     </row>
-    <row r="308" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="308" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A308">
         <v>14.1</v>
       </c>
@@ -9611,7 +9772,7 @@
         <v>9773.3678559927885</v>
       </c>
     </row>
-    <row r="309" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="309" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A309">
         <v>14.2</v>
       </c>
@@ -9640,7 +9801,7 @@
         <v>52863.766066058772</v>
       </c>
     </row>
-    <row r="310" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="310" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A310">
         <v>14.1</v>
       </c>
@@ -9669,7 +9830,7 @@
         <v>9869.3225420088074</v>
       </c>
     </row>
-    <row r="311" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="311" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A311">
         <v>14.2</v>
       </c>
@@ -9698,7 +9859,7 @@
         <v>53382.781225340077</v>
       </c>
     </row>
-    <row r="312" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="312" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A312">
         <v>14.1</v>
       </c>
@@ -9727,7 +9888,7 @@
         <v>9965.556064847844</v>
       </c>
     </row>
-    <row r="313" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="313" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A313">
         <v>14.2</v>
       </c>
@@ -9756,7 +9917,7 @@
         <v>53903.304602136559</v>
       </c>
     </row>
-    <row r="314" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="314" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A314">
         <v>14.1</v>
       </c>
@@ -9785,7 +9946,7 @@
         <v>10062.0684245099</v>
       </c>
     </row>
-    <row r="315" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="315" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A315">
         <v>14.2</v>
       </c>
@@ -9814,7 +9975,7 @@
         <v>54425.336196448203</v>
       </c>
     </row>
-    <row r="316" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="316" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A316">
         <v>14.1</v>
       </c>
@@ -9843,7 +10004,7 @@
         <v>10158.859620994959</v>
       </c>
     </row>
-    <row r="317" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="317" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A317">
         <v>14.2</v>
       </c>
@@ -9872,7 +10033,7 @@
         <v>54948.876008275001</v>
       </c>
     </row>
-    <row r="318" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="318" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A318">
         <v>14.1</v>
       </c>
@@ -9901,7 +10062,7 @@
         <v>10255.92965430305</v>
       </c>
     </row>
-    <row r="319" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="319" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A319">
         <v>14.2</v>
       </c>
@@ -9930,7 +10091,7 @@
         <v>55473.924037616962</v>
       </c>
     </row>
-    <row r="320" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="320" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A320">
         <v>14.1</v>
       </c>
@@ -9959,7 +10120,7 @@
         <v>10353.278524434139</v>
       </c>
     </row>
-    <row r="321" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="321" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A321">
         <v>14.2</v>
       </c>
@@ -9988,7 +10149,7 @@
         <v>56000.480284474063</v>
       </c>
     </row>
-    <row r="322" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="322" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A322">
         <v>14.1</v>
       </c>
@@ -10017,7 +10178,7 @@
         <v>9263.8859550375455</v>
       </c>
     </row>
-    <row r="323" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="323" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A323">
         <v>14.2</v>
       </c>
@@ -10046,7 +10207,7 @@
         <v>50107.998307816233</v>
       </c>
     </row>
-    <row r="324" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="324" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A324">
         <v>14.1</v>
       </c>
@@ -10075,7 +10236,7 @@
         <v>9334.0377977488515</v>
       </c>
     </row>
-    <row r="325" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="325" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A325">
         <v>14.2</v>
       </c>
@@ -10104,7 +10265,7 @@
         <v>50487.446892668122</v>
       </c>
     </row>
-    <row r="326" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="326" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A326">
         <v>14.1</v>
       </c>
@@ -10133,7 +10294,7 @@
         <v>9416.3276210569329</v>
       </c>
     </row>
-    <row r="327" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="327" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A327">
         <v>14.2</v>
       </c>
@@ -10162,7 +10323,7 @@
         <v>50932.549341800674</v>
       </c>
     </row>
-    <row r="328" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="328" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A328">
         <v>14.1</v>
       </c>
@@ -10191,7 +10352,7 @@
         <v>9506.0112118610195</v>
       </c>
     </row>
-    <row r="329" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="329" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A329">
         <v>14.2</v>
       </c>
@@ -10220,7 +10381,7 @@
         <v>51417.644391336173</v>
       </c>
     </row>
-    <row r="330" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="330" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A330">
         <v>14.1</v>
       </c>
@@ -10249,7 +10410,7 @@
         <v>9600.6705561847666</v>
       </c>
     </row>
-    <row r="331" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="331" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A331">
         <v>14.2</v>
       </c>
@@ -10278,7 +10439,7 @@
         <v>51929.65309785679</v>
       </c>
     </row>
-    <row r="332" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="332" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A332">
         <v>14.1</v>
       </c>
@@ -10307,7 +10468,7 @@
         <v>9699.0920645745646</v>
       </c>
     </row>
-    <row r="333" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="333" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A333">
         <v>14.2</v>
       </c>
@@ -10336,7 +10497,7 @@
         <v>52462.011203276568</v>
       </c>
     </row>
-    <row r="334" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="334" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A334">
         <v>14.1</v>
       </c>
@@ -10365,7 +10526,7 @@
         <v>9800.6858865173472</v>
       </c>
     </row>
-    <row r="335" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="335" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A335">
         <v>14.2</v>
       </c>
@@ -10394,7 +10555,7 @@
         <v>53011.528229144671</v>
       </c>
     </row>
-    <row r="336" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="336" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A336">
         <v>14.1</v>
       </c>
@@ -10423,7 +10584,7 @@
         <v>9905.1853205803909</v>
       </c>
     </row>
-    <row r="337" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="337" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A337">
         <v>14.2</v>
       </c>
@@ -10452,7 +10613,7 @@
         <v>53576.761597799363</v>
       </c>
     </row>
-    <row r="338" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="338" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A338">
         <v>14.1</v>
       </c>
@@ -10481,7 +10642,7 @@
         <v>10012.491216151881</v>
       </c>
     </row>
-    <row r="339" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="339" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A339">
         <v>14.2</v>
       </c>
@@ -10510,7 +10671,7 @@
         <v>54157.175007443213</v>
       </c>
     </row>
-    <row r="340" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="340" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A340">
         <v>14.1</v>
       </c>
@@ -10539,7 +10700,7 @@
         <v>10122.59142987548</v>
       </c>
     </row>
-    <row r="341" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="341" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A341">
         <v>14.2</v>
       </c>
@@ -10568,7 +10729,7 @@
         <v>54752.70277513472</v>
       </c>
     </row>
-    <row r="342" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="342" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A342">
         <v>14.3</v>
       </c>
@@ -10597,7 +10758,7 @@
         <v>56552.414086080753</v>
       </c>
     </row>
-    <row r="343" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="343" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A343">
         <v>14.4</v>
       </c>
@@ -10626,7 +10787,7 @@
         <v>4250.5326261078344</v>
       </c>
     </row>
-    <row r="344" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="344" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A344">
         <v>14.3</v>
       </c>
@@ -10655,7 +10816,7 @@
         <v>57119.407044400919</v>
       </c>
     </row>
-    <row r="345" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="345" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A345">
         <v>14.4</v>
       </c>
@@ -10684,7 +10845,7 @@
         <v>4293.1483500704726</v>
       </c>
     </row>
-    <row r="346" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="346" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A346">
         <v>14.3</v>
       </c>
@@ -10713,7 +10874,7 @@
         <v>57688.062130009188</v>
       </c>
     </row>
-    <row r="347" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="347" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A347">
         <v>14.4</v>
       </c>
@@ -10742,7 +10903,7 @@
         <v>4335.8890010831956</v>
       </c>
     </row>
-    <row r="348" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="348" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A348">
         <v>14.3</v>
       </c>
@@ -10771,7 +10932,7 @@
         <v>58258.379342905551</v>
       </c>
     </row>
-    <row r="349" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="349" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A349">
         <v>14.4</v>
       </c>
@@ -10800,7 +10961,7 @@
         <v>4378.7545791459988</v>
       </c>
     </row>
-    <row r="350" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="350" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A350">
         <v>14.3</v>
       </c>
@@ -10829,7 +10990,7 @@
         <v>58830.358683090002</v>
       </c>
     </row>
-    <row r="351" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="351" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A351">
         <v>14.4</v>
       </c>
@@ -10858,7 +11019,7 @@
         <v>4421.7450842588833</v>
       </c>
     </row>
-    <row r="352" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="352" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A352">
         <v>14.3</v>
       </c>
@@ -10887,7 +11048,7 @@
         <v>59404.000150562548</v>
       </c>
     </row>
-    <row r="353" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="353" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A353">
         <v>14.4</v>
       </c>
@@ -10916,7 +11077,7 @@
         <v>4464.8605164218507</v>
       </c>
     </row>
-    <row r="354" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="354" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A354">
         <v>14.3</v>
       </c>
@@ -10945,7 +11106,7 @@
         <v>59979.303745323188</v>
       </c>
     </row>
-    <row r="355" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="355" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A355">
         <v>14.4</v>
       </c>
@@ -10974,7 +11135,7 @@
         <v>4508.1008756348992</v>
       </c>
     </row>
-    <row r="356" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="356" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A356">
         <v>14.3</v>
       </c>
@@ -11003,7 +11164,7 @@
         <v>60556.269467371923</v>
       </c>
     </row>
-    <row r="357" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="357" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A357">
         <v>14.4</v>
       </c>
@@ -11032,7 +11193,7 @@
         <v>4551.4661618980308</v>
       </c>
     </row>
-    <row r="358" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="358" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A358">
         <v>14.3</v>
       </c>
@@ -11061,7 +11222,7 @@
         <v>61134.897316708753</v>
       </c>
     </row>
-    <row r="359" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="359" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A359">
         <v>14.4</v>
       </c>
@@ -11090,7 +11251,7 @@
         <v>4594.9563752112444</v>
       </c>
     </row>
-    <row r="360" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="360" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A360">
         <v>14.3</v>
       </c>
@@ -11119,7 +11280,7 @@
         <v>61715.187293333664</v>
       </c>
     </row>
-    <row r="361" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="361" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A361">
         <v>14.4</v>
       </c>
@@ -11148,7 +11309,7 @@
         <v>4638.5715155745374</v>
       </c>
     </row>
-    <row r="362" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="362" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A362">
         <v>14.3</v>
       </c>
@@ -11177,7 +11338,7 @@
         <v>55221.39247291936</v>
       </c>
     </row>
-    <row r="363" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="363" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A363">
         <v>14.4</v>
       </c>
@@ -11206,7 +11367,7 @@
         <v>4150.4917899344118</v>
       </c>
     </row>
-    <row r="364" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="364" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A364">
         <v>14.3</v>
       </c>
@@ -11235,7 +11396,7 @@
         <v>55639.562823662178</v>
       </c>
     </row>
-    <row r="365" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="365" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A365">
         <v>14.4</v>
       </c>
@@ -11264,7 +11425,7 @@
         <v>4181.9218667547893</v>
       </c>
     </row>
-    <row r="366" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="366" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A366">
         <v>14.3</v>
       </c>
@@ -11293,7 +11454,7 @@
         <v>56130.086849052597</v>
       </c>
     </row>
-    <row r="367" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="367" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A367">
         <v>14.4</v>
       </c>
@@ -11322,7 +11483,7 @@
         <v>4218.7901138050047</v>
       </c>
     </row>
-    <row r="368" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="368" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A368">
         <v>14.3</v>
       </c>
@@ -11351,7 +11512,7 @@
         <v>56664.68461830516</v>
       </c>
     </row>
-    <row r="369" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="369" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A369">
         <v>14.4</v>
       </c>
@@ -11380,7 +11541,7 @@
         <v>4258.9709848920229</v>
       </c>
     </row>
-    <row r="370" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="370" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A370">
         <v>14.3</v>
       </c>
@@ -11409,7 +11570,7 @@
         <v>57228.942514991417</v>
       </c>
     </row>
-    <row r="371" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="371" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A371">
         <v>14.4</v>
       </c>
@@ -11438,7 +11599,7 @@
         <v>4301.3811390501323</v>
       </c>
     </row>
-    <row r="372" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="372" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A372">
         <v>14.3</v>
       </c>
@@ -11467,7 +11628,7 @@
         <v>57815.626415133163</v>
       </c>
     </row>
-    <row r="373" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="373" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A373">
         <v>14.4</v>
       </c>
@@ -11496,7 +11657,7 @@
         <v>4345.4768527179676</v>
       </c>
     </row>
-    <row r="374" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="374" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A374">
         <v>14.3</v>
       </c>
@@ -11525,7 +11686,7 @@
         <v>58421.220260043949</v>
       </c>
     </row>
-    <row r="375" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="375" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A375">
         <v>14.4</v>
       </c>
@@ -11554,7 +11715,7 @@
         <v>4390.9938556180596</v>
       </c>
     </row>
-    <row r="376" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="376" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A376">
         <v>14.3</v>
       </c>
@@ -11583,7 +11744,7 @@
         <v>59044.134260669722</v>
       </c>
     </row>
-    <row r="377" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="377" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A377">
         <v>14.4</v>
       </c>
@@ -11612,7 +11773,7 @@
         <v>4437.8126577100284</v>
       </c>
     </row>
-    <row r="378" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="378" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A378">
         <v>14.3</v>
       </c>
@@ -11641,7 +11802,7 @@
         <v>59683.777386974543</v>
       </c>
     </row>
-    <row r="379" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="379" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A379">
         <v>14.4</v>
       </c>
@@ -11670,7 +11831,7 @@
         <v>4485.8888366205483</v>
       </c>
     </row>
-    <row r="380" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="380" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A380">
         <v>14.3</v>
       </c>
@@ -11699,7 +11860,7 @@
         <v>60340.077253239288</v>
       </c>
     </row>
-    <row r="381" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="381" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A381">
         <v>14.4</v>
       </c>
@@ -12018,7 +12179,7 @@
         <v>96.379082046683891</v>
       </c>
     </row>
-    <row r="392" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="392" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A392">
         <v>323</v>
       </c>
@@ -12047,7 +12208,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="393" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="393" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A393">
         <v>323</v>
       </c>
@@ -12076,7 +12237,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="394" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="394" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A394">
         <v>323</v>
       </c>
@@ -12105,7 +12266,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="395" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="395" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A395">
         <v>323</v>
       </c>
@@ -12134,7 +12295,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="396" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="396" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A396">
         <v>323</v>
       </c>
@@ -12163,7 +12324,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="397" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="397" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A397">
         <v>376</v>
       </c>
@@ -12192,7 +12353,7 @@
         <v>36033.446856183858</v>
       </c>
     </row>
-    <row r="398" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="398" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A398">
         <v>376</v>
       </c>
@@ -12221,7 +12382,7 @@
         <v>38872.61512155136</v>
       </c>
     </row>
-    <row r="399" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="399" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A399">
         <v>376</v>
       </c>
@@ -12250,7 +12411,7 @@
         <v>41717.57657108127</v>
       </c>
     </row>
-    <row r="400" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="400" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A400">
         <v>376</v>
       </c>
@@ -12279,7 +12440,7 @@
         <v>44568.331204773582</v>
       </c>
     </row>
-    <row r="401" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="401" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A401">
         <v>376</v>
       </c>
@@ -12308,7 +12469,7 @@
         <v>47424.879022628324</v>
       </c>
     </row>
-    <row r="402" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="402" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A402">
         <v>376</v>
       </c>
@@ -12337,7 +12498,7 @@
         <v>34556.673694232348</v>
       </c>
     </row>
-    <row r="403" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="403" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A403">
         <v>376</v>
       </c>
@@ -12366,7 +12527,7 @@
         <v>37856.02412414951</v>
       </c>
     </row>
-    <row r="404" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="404" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A404">
         <v>376</v>
       </c>
@@ -12395,7 +12556,7 @@
         <v>41689.182193960667</v>
       </c>
     </row>
-    <row r="405" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="405" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A405">
         <v>376</v>
       </c>
@@ -12424,7 +12585,7 @@
         <v>46057.780844716202</v>
       </c>
     </row>
-    <row r="406" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="406" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A406">
         <v>376</v>
       </c>
@@ -12453,7 +12614,7 @@
         <v>50963.453017466447</v>
       </c>
     </row>
-    <row r="407" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="407" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A407">
         <v>466</v>
       </c>
@@ -12482,7 +12643,7 @@
         <v>60.742268041340189</v>
       </c>
     </row>
-    <row r="408" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="408" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A408">
         <v>466</v>
       </c>
@@ -12511,7 +12672,7 @@
         <v>62.622639562581618</v>
       </c>
     </row>
-    <row r="409" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="409" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A409">
         <v>466</v>
       </c>
@@ -12540,7 +12701,7 @@
         <v>64.561276595843793</v>
       </c>
     </row>
-    <row r="410" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="410" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A410">
         <v>466</v>
       </c>
@@ -12569,7 +12730,7 @@
         <v>66.559986395217919</v>
       </c>
     </row>
-    <row r="411" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="411" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A411">
         <v>466</v>
       </c>
@@ -12598,7 +12759,7 @@
         <v>68.620632331635861</v>
       </c>
     </row>
-    <row r="412" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="412" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A412">
         <v>466</v>
       </c>
@@ -12627,7 +12788,7 @@
         <v>57.97444574550294</v>
       </c>
     </row>
-    <row r="413" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="413" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A413">
         <v>466</v>
       </c>
@@ -12656,7 +12817,7 @@
         <v>59.769135016331823</v>
       </c>
     </row>
-    <row r="414" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="414" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A414">
         <v>466</v>
       </c>
@@ -12685,7 +12846,7 @@
         <v>61.619434834385345</v>
       </c>
     </row>
-    <row r="415" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="415" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A415">
         <v>466</v>
       </c>
@@ -12714,7 +12875,7 @@
         <v>63.527070103221561</v>
       </c>
     </row>
-    <row r="416" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="416" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A416">
         <v>466</v>
       </c>
@@ -12743,7 +12904,7 @@
         <v>65.493819286181989</v>
       </c>
     </row>
-    <row r="417" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="417" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A417">
         <v>96</v>
       </c>
@@ -12772,7 +12933,7 @@
         <v>990.23735660954856</v>
       </c>
     </row>
-    <row r="418" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="418" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A418">
         <v>96</v>
       </c>
@@ -12801,7 +12962,7 @@
         <v>1074.101030045967</v>
       </c>
     </row>
-    <row r="419" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="419" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A419">
         <v>96</v>
       </c>
@@ -12830,7 +12991,7 @@
         <v>1165.04537214991</v>
       </c>
     </row>
-    <row r="420" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="420" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A420">
         <v>96</v>
       </c>
@@ -12859,7 +13020,7 @@
         <v>1263.666562398188</v>
       </c>
     </row>
-    <row r="421" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="421" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A421">
         <v>96</v>
       </c>
@@ -12888,7 +13049,7 @@
         <v>1370.6108527044289</v>
       </c>
     </row>
-    <row r="422" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="422" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A422">
         <v>385</v>
       </c>
@@ -12917,7 +13078,7 @@
         <v>22394.58706838209</v>
       </c>
     </row>
-    <row r="423" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="423" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A423">
         <v>385</v>
       </c>
@@ -12946,7 +13107,7 @@
         <v>24510.31089960839</v>
       </c>
     </row>
-    <row r="424" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="424" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A424">
         <v>385</v>
       </c>
@@ -12975,7 +13136,7 @@
         <v>26645.972550694249</v>
       </c>
     </row>
-    <row r="425" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="425" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A425">
         <v>385</v>
       </c>
@@ -13004,7 +13165,7 @@
         <v>28801.572021639651</v>
       </c>
     </row>
-    <row r="426" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="426" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A426">
         <v>385</v>
       </c>
@@ -13033,7 +13194,7 @@
         <v>30977.109312444602</v>
       </c>
     </row>
-    <row r="427" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="427" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A427">
         <v>385</v>
       </c>
@@ -13062,7 +13223,7 @@
         <v>20844.165363419648</v>
       </c>
     </row>
-    <row r="428" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="428" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A428">
         <v>385</v>
       </c>
@@ -13091,7 +13252,7 @@
         <v>22863.33165174054</v>
       </c>
     </row>
-    <row r="429" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="429" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A429">
         <v>385</v>
       </c>
@@ -13120,7 +13281,7 @@
         <v>25170.11368192935</v>
       </c>
     </row>
-    <row r="430" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="430" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A430">
         <v>385</v>
       </c>
@@ -13149,7 +13310,7 @@
         <v>27768.499991978719</v>
       </c>
     </row>
-    <row r="431" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="431" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A431">
         <v>385</v>
       </c>
@@ -13178,7 +13339,7 @@
         <v>30662.479119881289</v>
       </c>
     </row>
-    <row r="432" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="432" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A432" s="3">
         <v>386.1</v>
       </c>
@@ -13207,7 +13368,7 @@
         <v>6063.9485940000004</v>
       </c>
     </row>
-    <row r="433" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="433" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A433" s="3">
         <v>386.1</v>
       </c>
@@ -13236,7 +13397,7 @@
         <v>7617.8354212124996</v>
       </c>
     </row>
-    <row r="434" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="434" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A434" s="3">
         <v>386.1</v>
       </c>
@@ -13265,7 +13426,7 @@
         <v>9569.6688749062487</v>
       </c>
     </row>
-    <row r="435" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="435" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A435" s="3">
         <v>386.1</v>
       </c>
@@ -13294,7 +13455,7 @@
         <v>11023.172622260399</v>
       </c>
     </row>
-    <row r="436" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="436" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A436" s="3">
         <v>386.1</v>
       </c>
@@ -13323,7 +13484,7 @@
         <v>12345.410811333601</v>
       </c>
     </row>
-    <row r="437" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="437" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A437" s="3">
         <v>386.2</v>
       </c>
@@ -13352,7 +13513,7 @@
         <v>7569.1213256024957</v>
       </c>
     </row>
-    <row r="438" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="438" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A438" s="3">
         <v>386.2</v>
       </c>
@@ -13381,7 +13542,7 @@
         <v>7660.696088310985</v>
       </c>
     </row>
-    <row r="439" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="439" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A439" s="3">
         <v>386.2</v>
       </c>
@@ -13410,7 +13571,7 @@
         <v>7752.6631555816357</v>
       </c>
     </row>
-    <row r="440" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="440" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A440" s="3">
         <v>386.2</v>
       </c>
@@ -13439,7 +13600,7 @@
         <v>7845.0225274144459</v>
       </c>
     </row>
-    <row r="441" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="441" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A441" s="3">
         <v>386.2</v>
       </c>
@@ -13468,7 +13629,7 @@
         <v>7937.7742038094157</v>
       </c>
     </row>
-    <row r="442" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="442" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A442" s="3">
         <v>386.3</v>
       </c>
@@ -13497,7 +13658,7 @@
         <v>7026.0817481999993</v>
       </c>
     </row>
-    <row r="443" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="443" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A443" s="3">
         <v>386.3</v>
       </c>
@@ -13526,7 +13687,7 @@
         <v>7738.846362034199</v>
       </c>
     </row>
-    <row r="444" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="444" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A444" s="3">
         <v>386.3</v>
       </c>
@@ -13555,7 +13716,7 @@
         <v>8458.3536047747984</v>
       </c>
     </row>
-    <row r="445" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="445" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A445" s="3">
         <v>386.3</v>
       </c>
@@ -13584,7 +13745,7 @@
         <v>9184.6034764218002</v>
       </c>
     </row>
-    <row r="446" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="446" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A446" s="3">
         <v>386.3</v>
       </c>
@@ -13613,7 +13774,7 @@
         <v>9917.5959769751989</v>
       </c>
     </row>
-    <row r="447" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="447" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A447" t="s">
         <v>68</v>
       </c>
@@ -13642,7 +13803,7 @@
         <v>16.2</v>
       </c>
     </row>
-    <row r="448" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="448" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A448" t="s">
         <v>68</v>
       </c>
@@ -13671,7 +13832,7 @@
         <v>16.8</v>
       </c>
     </row>
-    <row r="449" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="449" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A449" t="s">
         <v>68</v>
       </c>
@@ -13700,7 +13861,7 @@
         <v>17.3</v>
       </c>
     </row>
-    <row r="450" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="450" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A450" t="s">
         <v>68</v>
       </c>
@@ -13729,7 +13890,7 @@
         <v>17.899999999999999</v>
       </c>
     </row>
-    <row r="451" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="451" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A451" t="s">
         <v>68</v>
       </c>
@@ -13758,7 +13919,7 @@
         <v>18.3</v>
       </c>
     </row>
-    <row r="452" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="452" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A452" t="s">
         <v>68</v>
       </c>
@@ -13787,7 +13948,7 @@
         <v>16.2</v>
       </c>
     </row>
-    <row r="453" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="453" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A453" t="s">
         <v>68</v>
       </c>
@@ -13816,7 +13977,7 @@
         <v>16.8</v>
       </c>
     </row>
-    <row r="454" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="454" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A454" t="s">
         <v>68</v>
       </c>
@@ -13845,7 +14006,7 @@
         <v>17.3</v>
       </c>
     </row>
-    <row r="455" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="455" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A455" t="s">
         <v>68</v>
       </c>
@@ -13874,7 +14035,7 @@
         <v>17.899999999999999</v>
       </c>
     </row>
-    <row r="456" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="456" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A456" t="s">
         <v>68</v>
       </c>
@@ -13903,7 +14064,7 @@
         <v>18.2</v>
       </c>
     </row>
-    <row r="457" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="457" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A457" t="s">
         <v>69</v>
       </c>
@@ -13932,7 +14093,7 @@
         <v>41.957999999999991</v>
       </c>
     </row>
-    <row r="458" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="458" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A458" t="s">
         <v>69</v>
       </c>
@@ -13961,7 +14122,7 @@
         <v>44.276179499999998</v>
       </c>
     </row>
-    <row r="459" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="459" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A459" t="s">
         <v>69</v>
       </c>
@@ -13990,7 +14151,7 @@
         <v>46.721281949999991</v>
       </c>
     </row>
-    <row r="460" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="460" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A460" t="s">
         <v>69</v>
       </c>
@@ -14019,7 +14180,7 @@
         <v>49.300204196249993</v>
       </c>
     </row>
-    <row r="461" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="461" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A461" t="s">
         <v>69</v>
       </c>
@@ -14048,7 +14209,7 @@
         <v>52.020215462249993</v>
       </c>
     </row>
-    <row r="462" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="462" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A462">
         <v>332</v>
       </c>
@@ -14077,7 +14238,7 @@
         <v>0.69049565217391329</v>
       </c>
     </row>
-    <row r="463" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="463" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A463">
         <v>332</v>
       </c>
@@ -14106,7 +14267,7 @@
         <v>0.61943446956521764</v>
       </c>
     </row>
-    <row r="464" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="464" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A464">
         <v>332</v>
       </c>
@@ -14135,7 +14296,7 @@
         <v>0.5556805669565219</v>
       </c>
     </row>
-    <row r="465" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="465" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A465">
         <v>332</v>
       </c>
@@ -14164,7 +14325,7 @@
         <v>0.49848310017391317</v>
       </c>
     </row>
-    <row r="466" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="466" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A466">
         <v>332</v>
       </c>
@@ -14194,6 +14355,13 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:K466" xr:uid="{52F5ABF9-7414-4626-A0F7-29EA0F0D3250}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="194"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>